<commit_message>
Updated Customer Contact Sheet
</commit_message>
<xml_diff>
--- a/Reference Data/XLSX Workbooks/Customer Information.xlsx
+++ b/Reference Data/XLSX Workbooks/Customer Information.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E155"/>
+  <dimension ref="A1:E154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3868,22 +3868,22 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Williams</t>
+          <t>Z Constructors</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Station 150</t>
+          <t>Auto Park Dallas</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/kaxyjgx5dcjqozysedsvw/AGutILn_Cw8siidIM1J_vvI?rlkey=5mynmrgcc7fvyy35k3b8o1waq&amp;st=32gshoxy&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/hc5d0ky6qbgspofbonhuh/AGYaHMGsFj28vK4I9JW_gYw?rlkey=njykoxd52clgz3mvcluhic8b7&amp;st=swwsax4n&amp;dl=0</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>leann.sprayberry@williams.com, steven.johnston@williams.com, ssluttersr@gmail.com, james.a.raschke@williams.com,  bradley.george@williams.com, chad.dlugoszewski@williams.com, jeff.l.gallimore@williams.com, timothy.petrea@williams.com</t>
+          <t>mmccarter@zconstructors.com, tgeorge@zconstructors.com, cbowles@zconstructors.com, JLeckie@zconstructors.com</t>
         </is>
       </c>
     </row>
@@ -3895,17 +3895,17 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Auto Park Dallas</t>
+          <t>HG Supply Co</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/hc5d0ky6qbgspofbonhuh/AGYaHMGsFj28vK4I9JW_gYw?rlkey=njykoxd52clgz3mvcluhic8b7&amp;st=swwsax4n&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/2jneqj2ineo6rao3wlbgc/ALfEbccOU-r25SSqGpG-Ee0?rlkey=34gdlm0h577b5auv079zwap7k&amp;st=f8vdhybi&amp;dl=0</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>mmccarter@zconstructors.com, tgeorge@zconstructors.com, cbowles@zconstructors.com, JLeckie@zconstructors.com</t>
+          <t>cwest@zconstructors.com, JLeckie@zconstructors.com, jlanier@zconstructors.com, smcgaha@zconstructors.com</t>
         </is>
       </c>
     </row>
@@ -3917,17 +3917,17 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>HG Supply Co</t>
+          <t>Lowe Tractor Dealership</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/2jneqj2ineo6rao3wlbgc/ALfEbccOU-r25SSqGpG-Ee0?rlkey=34gdlm0h577b5auv079zwap7k&amp;st=f8vdhybi&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/fiyw8k18de2qtn2iz8qzz/AM3As2ii9Wjs3sqsNZ4d4y0?rlkey=z7cmn9ricob2mzxjl6w6kgq27&amp;st=hu8ngzc3&amp;dl=0</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>cwest@zconstructors.com, JLeckie@zconstructors.com, jlanier@zconstructors.com, smcgaha@zconstructors.com</t>
+          <t>Mwiskur@zconstructors.com, Cfloyd@zconstructors.com, JLeckie@zconstructors.com, jherron@zconstructors.com</t>
         </is>
       </c>
     </row>
@@ -3939,17 +3939,17 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Lowe Tractor Dealership</t>
+          <t>Quality Collision Fort Worth</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/fiyw8k18de2qtn2iz8qzz/AM3As2ii9Wjs3sqsNZ4d4y0?rlkey=z7cmn9ricob2mzxjl6w6kgq27&amp;st=hu8ngzc3&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/2u8zrjnonyi8ygmxv7mt9/AOEkPaYWXz8mWV-YBqyGXOQ?rlkey=mw1wcqb54u4uvo0npnx909n94&amp;st=2fds3bt3&amp;dl=0</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Mwiskur@zconstructors.com, Cfloyd@zconstructors.com, JLeckie@zconstructors.com, jherron@zconstructors.com</t>
+          <t>cwest@zconstructors.com, tdossett@zconstructors.com, JLeckie@zconstructors.com</t>
         </is>
       </c>
     </row>
@@ -3961,17 +3961,17 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Quality Collision Fort Worth</t>
+          <t>Quality Collision The Colony</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/2u8zrjnonyi8ygmxv7mt9/AOEkPaYWXz8mWV-YBqyGXOQ?rlkey=mw1wcqb54u4uvo0npnx909n94&amp;st=2fds3bt3&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/ec52f6ln5fznmlv6g2vot/AG49CtbntZ9XYgpF896wf20?rlkey=slbs0se42ejrlkoyvh5vj7tif&amp;st=ipbxcfkb&amp;dl=0</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>cwest@zconstructors.com, tdossett@zconstructors.com, JLeckie@zconstructors.com</t>
+          <t>cwest@zconstructors.com, JLeckie@zconstructors.com, smcgaha@zconstructors.com, jherron@zconstructors.com</t>
         </is>
       </c>
     </row>
@@ -3983,37 +3983,15 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Quality Collision The Colony</t>
+          <t>The Hub of Rowlett</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/ec52f6ln5fznmlv6g2vot/AG49CtbntZ9XYgpF896wf20?rlkey=slbs0se42ejrlkoyvh5vj7tif&amp;st=ipbxcfkb&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/fw05xwmsrzilkxvt83egu/AFl_XVDCw9aaCluq12G2Ky8?rlkey=0u77hgrf9kv7y392y7e4rmckb&amp;st=kftl8yme&amp;dl=0</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
-        <is>
-          <t>cwest@zconstructors.com, JLeckie@zconstructors.com, smcgaha@zconstructors.com, jherron@zconstructors.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>Z Constructors</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>The Hub of Rowlett</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/fw05xwmsrzilkxvt83egu/AFl_XVDCw9aaCluq12G2Ky8?rlkey=0u77hgrf9kv7y392y7e4rmckb&amp;st=kftl8yme&amp;dl=0</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
         <is>
           <t>cwest@zconstructors.com, jlanier@zconstructors.com, JLeckie@zconstructors.com, smcgaha@zconstructors.com</t>
         </is>
@@ -4031,7 +4009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78.42578125" customWidth="1" min="1" max="2"/>
@@ -4067,6 +4045,15 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -4438,6 +4425,116 @@
       <c r="D32" t="inlineStr">
         <is>
           <t>Mike.Smitherman@Williams.com, Roy.Guerrero@williams.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Station 145</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/z8kvz6pb2j2r09oo2c97g/AFQLt9GkR8taMaiVPmxvHh4?rlkey=4ts1b97rjx5lbe0br3fbc2wjf&amp;st=ru4xwzl3&amp;dl=0</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>joshua.colombo@williams.com, james.a.raschke@williams.com, Jeff.King@Williams.com, jeff.l.gallimore@williams.com, Sam.Lawrence@Williams.com, Kevin.Murray@Williams.com, chad.dlugoszewski@williams.com, Philip.Giblin@williams.com, Michael.T.Barron@Williams.com, Austin.Justice@williams.com, timothy.petrea@williams.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Station 150</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/kaxyjgx5dcjqozysedsvw/AGutILn_Cw8siidIM1J_vvI?rlkey=5mynmrgcc7fvyy35k3b8o1waq&amp;st=32gshoxy&amp;dl=0</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>leann.sprayberry@williams.com, steven.johnston@williams.com, ssluttersr@gmail.com, james.a.raschke@williams.com, bradley.george@williams.com, chad.dlugoszewski@williams.com, jeff.l.gallimore@williams.com, timothy.petrea@williams.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Station 155</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/m3ziycemltti4rntzjwxn/AAD0779D_F1HEl9iia9r07M?rlkey=2brdm1ebw4h6v4fx3gk0fbqvq&amp;st=4kae51wa&amp;dl=0</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>james.a.raschke@williams.com, leann.sprayberry@williams.com, steven.johnston@williams.com, ssluttersr@gmail.com, bradley.george@williams.com, keith.murray@williams.com, scott.emerson@williams.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Station 160</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/83sgdjxpgsdrnqdv8srm3/ADhvHR96Uyk1p8Ii4cNtouA?rlkey=o7d5rrmbpg7tgmedpsmb6owny&amp;st=fl56lkhe&amp;dl=0</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>james.a.raschke@williams.com, leann.sprayberry@williams.com, steven.johnston@williams.com, ssluttersr@gmail.com, bradley.george@williams.com, keith.murray@williams.com, scott.emerson@williams.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Station 165</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/7e1548qjcwrxwufynwox3/ANTe2IBK5ChXU-pU8cg42A8?rlkey=n023itk90g2p7tflky6pnp3os&amp;st=oz50awuz&amp;dl=0</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>joshua.colombo@williams.com, james.a.raschke@williams.com, Jeff.King@Williams.com, jeff.l.gallimore@williams.com, Sam.Lawrence@Williams.com, Kevin.Murray@Williams.com, chad.dlugoszewski@williams.com, Philip.Giblin@williams.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Conversion script for downloaded signature EML files
</commit_message>
<xml_diff>
--- a/Reference Data/XLSX Workbooks/Customer Information.xlsx
+++ b/Reference Data/XLSX Workbooks/Customer Information.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F119"/>
+  <dimension ref="A1:F118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2217,49 +2217,44 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Chambers County Justice Center</t>
+          <t>Montgomery County Mental Health Treatment Facility</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/9yksjubv94yr5wbu1f80t/APweuR7mw621WYxZ-8rBWR0?rlkey=l2wjt0a9alatgmnacnkj03j9k&amp;st=hzt8gnf3&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/ncmouccbszquodnj2a2rs/ACbyykpybiPXdJJvDN2JT_I?rlkey=ycssac5p0d0scs81rj0ui5l4u&amp;st=uvka754j&amp;dl=0</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>bchobot@satpon.com, jcervantes@satpon.com, dbihn@satpon.com, mrasmussen@satpon.com, aguerrero@satpon.com, pball@satpon.com, jshepherd@satpon.com, tgranato@satpon.com</t>
+          <t>bchobot@satpon.com, abeck@satpon.com, dwitte@satpon.com, smorris@satpon.com, scrozier@satpon.com, jbrooks@satpon.com</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/19ja32kmfghcbjxrgzpco/AEMXdgEtC985yTE-xR25oK8?rlkey=r2iz880hojxs7kdoz1xjnmg72&amp;st=o3nxotzq&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/avkpve5i28ik5sjqxroh9/APuoJbqWyg9csrPJzYSamLM?rlkey=mpm49lykc1kbc19699bmujiwf&amp;st=slhu2o6z&amp;dl=0</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Satterfield &amp; Pontikes</t>
+          <t>Schwob</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Montgomery County Mental Health Treatment Facility</t>
+          <t>AAA Cooper Fort Worth</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/ncmouccbszquodnj2a2rs/ACbyykpybiPXdJJvDN2JT_I?rlkey=ycssac5p0d0scs81rj0ui5l4u&amp;st=uvka754j&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/q6fflr83k4ux2r7r6xzih/AKcIsPQN6Q_fnBSypPNZpmU?rlkey=xcume6ont4ra3wgm5nvct224g&amp;st=lotnpsgr&amp;dl=0</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>bchobot@satpon.com, abeck@satpon.com, dwitte@satpon.com, smorris@satpon.com, scrozier@satpon.com, jbrooks@satpon.com</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/avkpve5i28ik5sjqxroh9/APuoJbqWyg9csrPJzYSamLM?rlkey=mpm49lykc1kbc19699bmujiwf&amp;st=slhu2o6z&amp;dl=0</t>
+          <t>rkorthauer@schwob.com, Jelliott@schwob.com, cbeasley@schwob.com</t>
         </is>
       </c>
     </row>
@@ -2271,17 +2266,22 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>AAA Cooper Fort Worth</t>
+          <t>Averitt Express OKC</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/q6fflr83k4ux2r7r6xzih/AKcIsPQN6Q_fnBSypPNZpmU?rlkey=xcume6ont4ra3wgm5nvct224g&amp;st=lotnpsgr&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/4y507x2schq2rahipegz1/AACWX9aur2ttwQ5_5M6iR4s?rlkey=lr3373tkteszw5sszb1yman02&amp;st=rfsni6l8&amp;dl=0</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>rkorthauer@schwob.com, Jelliott@schwob.com, cbeasley@schwob.com</t>
+          <t>rsnyder@schwob.com, cmartin@schwob.com, bwilde@schwob.com</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/dvsoajgo02bho8b7ajch4/AK0t0Y4rT0dHSObCjRh46J4?rlkey=dtp9swc3t9jtgi248dywk4b72&amp;st=q0y0l0iw&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2293,22 +2293,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Averitt Express OKC</t>
+          <t>Avis</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/4y507x2schq2rahipegz1/AACWX9aur2ttwQ5_5M6iR4s?rlkey=lr3373tkteszw5sszb1yman02&amp;st=rfsni6l8&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/uuxysiku8k8v0t6iyep6d/AOLjGY_IzxdGLTekr8I4acs?rlkey=f3vw1qh3lva2vt32k7nepxszp&amp;st=k9cj7265&amp;dl=0</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>rsnyder@schwob.com, cmartin@schwob.com, bwilde@schwob.com</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/dvsoajgo02bho8b7ajch4/AK0t0Y4rT0dHSObCjRh46J4?rlkey=dtp9swc3t9jtgi248dywk4b72&amp;st=q0y0l0iw&amp;dl=0</t>
+          <t>lgee@schwob.com, Cbeasley@schwob.com, Jmaxton@schwob.com</t>
         </is>
       </c>
     </row>
@@ -2320,17 +2315,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Avis</t>
+          <t>Inland Truck Parts Facility</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/uuxysiku8k8v0t6iyep6d/AOLjGY_IzxdGLTekr8I4acs?rlkey=f3vw1qh3lva2vt32k7nepxszp&amp;st=k9cj7265&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/hfsm41icyvt69qkajcbc9/AItxiV2LTYnGsiDMfz5rj8s?rlkey=hd07vio28gf3iizndqhr3wj4h&amp;st=pxl1utam&amp;dl=0</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>lgee@schwob.com, Cbeasley@schwob.com, Jmaxton@schwob.com</t>
+          <t>Jelliott@schwob.com, pmurphy@schwob.com, eknott@schwob.com</t>
         </is>
       </c>
     </row>
@@ -2342,17 +2337,22 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Inland Truck Parts Facility</t>
+          <t>Kiewit Maintenance Facility - Mebane</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/hfsm41icyvt69qkajcbc9/AItxiV2LTYnGsiDMfz5rj8s?rlkey=hd07vio28gf3iizndqhr3wj4h&amp;st=pxl1utam&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/hhnofk9b9er173gyyewly/ADyJ2k81Tjp8JwaW3qJMgrI?rlkey=0bxy30962tdxdqmjxbusw1yrf&amp;st=2kf4dh6h&amp;dl=0</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Jelliott@schwob.com, pmurphy@schwob.com, eknott@schwob.com</t>
+          <t>eknott@schwob.com, lgee@schwob.com, erush@schwob.com</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/cmwfybptmlen8dmkwcxrv/AO-HeXu6fzhUZsJWsyR8Nr4?rlkey=17yi7z9qu9nb8hz0dk1ixogzx&amp;st=jitgv1uz&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2364,22 +2364,22 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Kiewit Maintenance Facility - Mebane</t>
+          <t>SAIA Omaha</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/hhnofk9b9er173gyyewly/ADyJ2k81Tjp8JwaW3qJMgrI?rlkey=0bxy30962tdxdqmjxbusw1yrf&amp;st=2kf4dh6h&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/fmflvz9r57dodyg9m1wxs/AIKothjHquqjHAX__UWYnxY?rlkey=ua3cxy297qf29iut9ebbut4lx&amp;st=epk6j0yl&amp;dl=0</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>eknott@schwob.com, lgee@schwob.com, erush@schwob.com</t>
+          <t>MStieber@schwob.com, Eknott@schwob.com, abattard@schwob.com</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/cmwfybptmlen8dmkwcxrv/AO-HeXu6fzhUZsJWsyR8Nr4?rlkey=17yi7z9qu9nb8hz0dk1ixogzx&amp;st=jitgv1uz&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/t0ixtmdbw22dxf5oji397/ADK7qlce4twSYdCHV7oFogU?rlkey=wtxb11zpzjz9xvdi52mex4j73&amp;st=7jjnfxcg&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2391,22 +2391,22 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SAIA Omaha</t>
+          <t>SEFL Dallas</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/fmflvz9r57dodyg9m1wxs/AIKothjHquqjHAX__UWYnxY?rlkey=ua3cxy297qf29iut9ebbut4lx&amp;st=epk6j0yl&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/qvxa6jgfourgt9y3hqyv7/ALanIo1QftjDFRriGe1XoNg?rlkey=k2kszqem21qcty8ba4xguqbd1&amp;st=0aeaypil&amp;dl=0</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>MStieber@schwob.com, Eknott@schwob.com, abattard@schwob.com</t>
+          <t>rsnyder@schwob.com, mstieber@schwob.com</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/t0ixtmdbw22dxf5oji397/ADK7qlce4twSYdCHV7oFogU?rlkey=wtxb11zpzjz9xvdi52mex4j73&amp;st=7jjnfxcg&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/25tfe6sjr9579766xj3w8/AHSgOG0IieeBQtb500D4sko?rlkey=kaa9u00xaa1ap2vdqolqov4m7&amp;st=wqu7lbyc&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2418,22 +2418,22 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SEFL Dallas</t>
+          <t>SEFL Garland</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/qvxa6jgfourgt9y3hqyv7/ALanIo1QftjDFRriGe1XoNg?rlkey=k2kszqem21qcty8ba4xguqbd1&amp;st=0aeaypil&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/9tgx66ja5ika3b0374mo3/AMLDkPSZhID6ZWAyCMCwhB0?rlkey=tonjmf5j6znrt8bmzr95xecws&amp;st=okioei7l&amp;dl=0</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>rsnyder@schwob.com, mstieber@schwob.com</t>
+          <t>eknott@schwob.com, jmaxton@schwob.com</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/25tfe6sjr9579766xj3w8/AHSgOG0IieeBQtb500D4sko?rlkey=kaa9u00xaa1ap2vdqolqov4m7&amp;st=wqu7lbyc&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/djw7mvjkq2onpoaa1k5ao/AAXKqndlcAksIFd5kNGKXIw?rlkey=7rbciutymc0isshrnsszq6p7o&amp;st=l27n7wso&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SEFL Garland</t>
+          <t>SEFL Laredo</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/9tgx66ja5ika3b0374mo3/AMLDkPSZhID6ZWAyCMCwhB0?rlkey=tonjmf5j6znrt8bmzr95xecws&amp;st=okioei7l&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/chl9a07sgtq4y7fn01qov/ACbMw231bpmNkEMztVurfbc?rlkey=bzka0txpurw5qzyo28j46kb68&amp;st=evxkg9z1&amp;dl=0</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>eknott@schwob.com, jmaxton@schwob.com</t>
+          <t>ttaylor@schwob.com</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/djw7mvjkq2onpoaa1k5ao/AAXKqndlcAksIFd5kNGKXIw?rlkey=7rbciutymc0isshrnsszq6p7o&amp;st=l27n7wso&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/exgx4njf9esedqcv4gd9q/AMoAKMIcutIImDLxn1hE1gc?rlkey=ekeylz61mt6rakmf0c69kek1e&amp;st=fz5yrtn2&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2472,22 +2472,22 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SEFL Laredo</t>
+          <t>SEFL Shreveport</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/chl9a07sgtq4y7fn01qov/ACbMw231bpmNkEMztVurfbc?rlkey=bzka0txpurw5qzyo28j46kb68&amp;st=evxkg9z1&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/j5wk3bil5ll5jz1haqp0j/AEQH8kQhGJxb5raXZ-7Bve8?rlkey=wttaceyo1npi1pucejll7tenx&amp;st=x16rvwf8&amp;dl=0</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>ttaylor@schwob.com</t>
+          <t>rkorthauer@schwob.com, RSnyder@schwob.com</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/exgx4njf9esedqcv4gd9q/AMoAKMIcutIImDLxn1hE1gc?rlkey=ekeylz61mt6rakmf0c69kek1e&amp;st=fz5yrtn2&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/g6w596i9j2peapys18zr6/ADcBnQtpqV8xZysm4vSN2HI?rlkey=1evxsc2pbrwcpip1zxwvdzksx&amp;st=jaes60bl&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2499,49 +2499,44 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SEFL Shreveport</t>
+          <t>SEFL Van Buren</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/j5wk3bil5ll5jz1haqp0j/AEQH8kQhGJxb5raXZ-7Bve8?rlkey=wttaceyo1npi1pucejll7tenx&amp;st=x16rvwf8&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/3xe5wwvihqrmqongxb6kr/AE6WJwJ1ZN7CmJf6bOs71wI?rlkey=etdgnz2c87dn7xuy0vmxnbn2k&amp;st=81hwm5yl&amp;dl=0</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>rkorthauer@schwob.com, RSnyder@schwob.com</t>
+          <t>rkorthauer@schwob.com,</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/g6w596i9j2peapys18zr6/ADcBnQtpqV8xZysm4vSN2HI?rlkey=1evxsc2pbrwcpip1zxwvdzksx&amp;st=jaes60bl&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/msj6bv6s0znjrmtpbz27z/AIoVp38WZYhk5_CeOUOFaJ8?rlkey=fpbv771o4olqthznso3cypn5d&amp;st=igxdess9&amp;dl=0</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Schwob</t>
+          <t>Skiles Group</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SEFL Van Buren</t>
+          <t>Olney Hamilton Hospital</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/3xe5wwvihqrmqongxb6kr/AE6WJwJ1ZN7CmJf6bOs71wI?rlkey=etdgnz2c87dn7xuy0vmxnbn2k&amp;st=81hwm5yl&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/ofo0se1ajznij6rvapqho/ABv7YSIUOyoZVDwlIEiLkcA?rlkey=r06imgcm7ljqxdq3plrbf1xko&amp;st=y7c5hqjm&amp;dl=0</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>rkorthauer@schwob.com,</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/msj6bv6s0znjrmtpbz27z/AIoVp38WZYhk5_CeOUOFaJ8?rlkey=fpbv771o4olqthznso3cypn5d&amp;st=igxdess9&amp;dl=0</t>
+          <t>zwymer@skilesgroup.com, tdougherty@skilesgroup.com, jtribble@skilesgroup.com</t>
         </is>
       </c>
     </row>
@@ -2553,39 +2548,44 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Olney Hamilton Hospital</t>
+          <t>THR Midlothian</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/ofo0se1ajznij6rvapqho/ABv7YSIUOyoZVDwlIEiLkcA?rlkey=r06imgcm7ljqxdq3plrbf1xko&amp;st=y7c5hqjm&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/tww7deesvod5g3ejk68sj/AOxnL35T6a-tUvA1qdxeM78?rlkey=2nautjorvodan3t4jqieynapy&amp;st=40glc2w3&amp;dl=0</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>zwymer@skilesgroup.com, tdougherty@skilesgroup.com, jtribble@skilesgroup.com</t>
+          <t>cdeshong@skilesgroup.com, prose@skilesgroup.com</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Skiles Group</t>
+          <t>Spring Valley</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>THR Midlothian</t>
+          <t>Brandon Industries</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/tww7deesvod5g3ejk68sj/AOxnL35T6a-tUvA1qdxeM78?rlkey=2nautjorvodan3t4jqieynapy&amp;st=40glc2w3&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/jew555qn3ibymcby9jp1n/APW-Gstq5rbtuP8QmiNes18?rlkey=psfseu3fcaxt8s3zu1ntg3f41&amp;st=yi9mu5l4&amp;dl=0</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>cdeshong@skilesgroup.com, prose@skilesgroup.com</t>
+          <t>Dbyrnes@svcc.biz, Wcaddell@svcc.biz, cvargas@svcc.biz</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>https://app.procore.com/webclients/host/companies/29589/projects/2839213/tools/photos/albums/20423147?page=1&amp;sort=-exposure_date</t>
         </is>
       </c>
     </row>
@@ -2597,22 +2597,27 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Brandon Industries</t>
+          <t>Hughes House 3</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/jew555qn3ibymcby9jp1n/APW-Gstq5rbtuP8QmiNes18?rlkey=psfseu3fcaxt8s3zu1ntg3f41&amp;st=yi9mu5l4&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/vpjclef84oxn3ujcdm7oq/AMj4y1IPfN9Nsltr5XQ42AI?rlkey=xsyol3tx830bxysnpvkzgqfnr&amp;st=cam4njgk&amp;dl=0</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Dbyrnes@svcc.biz, Wcaddell@svcc.biz, cvargas@svcc.biz</t>
+          <t>sstackenwalt@svcc.biz, wcaddell@svcc.biz, cvargas@svcc.biz</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>https://app.procore.com/webclients/host/companies/29589/projects/2839213/tools/photos/albums/20423147?page=1&amp;sort=-exposure_date</t>
+          <t>https://app.procore.com/webclients/host/companies/29589/projects/3075405/tools/photos/albums/19460376?page=1&amp;sort=-exposure_date</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/xkrmq5pajmtsp8dyk8215/AFLz4hX89up39PwluPqOc1I?rlkey=2ripaid2chklc0yi5x1n5v91x&amp;st=3ys0p7qp&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2624,27 +2629,27 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Hughes House 3</t>
+          <t>Juliette Fowler Demo &amp; Reno</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/vpjclef84oxn3ujcdm7oq/AMj4y1IPfN9Nsltr5XQ42AI?rlkey=xsyol3tx830bxysnpvkzgqfnr&amp;st=cam4njgk&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/f8pg4n8oudwjn88qegnwh/AGSsmOTZ48-qJHTe1-W2_lo?rlkey=e4afo4ltzd40tsm4mlq0s8njj&amp;st=bqvmugh9&amp;dl=0</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>sstackenwalt@svcc.biz, wcaddell@svcc.biz, cvargas@svcc.biz</t>
+          <t>rgartner@svcc.biz, wcaddell@svcc.biz, tholt@svcc.biz, nicoleg@fowlercommunities.org, larryh@fowlercommunities.org, cvargas@svcc.biz</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>https://app.procore.com/webclients/host/companies/29589/projects/3075405/tools/photos/albums/19460376?page=1&amp;sort=-exposure_date</t>
+          <t>https://app.procore.com/1340278/project/images/albums?page=1&amp;sort=-exposure_date</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/xkrmq5pajmtsp8dyk8215/AFLz4hX89up39PwluPqOc1I?rlkey=2ripaid2chklc0yi5x1n5v91x&amp;st=3ys0p7qp&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/9jvmr6dz5fakocf30cw4b/AKlU6hlDLL9d0poXlhfTowY?rlkey=dryyheuisxdde193cvhtvmuns&amp;st=ev82vu17&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2656,27 +2661,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Juliette Fowler Demo &amp; Reno</t>
+          <t>Juliette Fowler Phase 2 Ebby House</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/f8pg4n8oudwjn88qegnwh/AGSsmOTZ48-qJHTe1-W2_lo?rlkey=e4afo4ltzd40tsm4mlq0s8njj&amp;st=bqvmugh9&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/kr0p43hzsolafl9eo07r3/ADrBTKolqI4D_Qf9e_XSbnU?rlkey=dur7d3er0gbhsy8qq8ugd2fyj&amp;st=jap9kq4n&amp;dl=0</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>rgartner@svcc.biz, wcaddell@svcc.biz, tholt@svcc.biz, nicoleg@fowlercommunities.org, larryh@fowlercommunities.org, cvargas@svcc.biz</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>https://app.procore.com/1340278/project/images/albums?page=1&amp;sort=-exposure_date</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/9jvmr6dz5fakocf30cw4b/AKlU6hlDLL9d0poXlhfTowY?rlkey=dryyheuisxdde193cvhtvmuns&amp;st=ev82vu17&amp;dl=0</t>
+          <t>Rgartner@svcc.biz, tholt@svcc.biz, wcaddell@svcc.biz, cvargas@svcc.biz</t>
         </is>
       </c>
     </row>
@@ -2688,17 +2683,22 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Juliette Fowler Phase 2 Ebby House</t>
+          <t>Meals on Wheels</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/kr0p43hzsolafl9eo07r3/ADrBTKolqI4D_Qf9e_XSbnU?rlkey=dur7d3er0gbhsy8qq8ugd2fyj&amp;st=jap9kq4n&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/k1x3uhhsva3llk0r1vdxw/ADzOeKbPDUWS9rhgBWox-1M?rlkey=4u6z93o1v19wo5bqrdt62soig&amp;st=5q9fupd8&amp;dl=0</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Rgartner@svcc.biz, tholt@svcc.biz, wcaddell@svcc.biz, cvargas@svcc.biz</t>
+          <t>cvargas@svcc.biz, kvirant@svcc.biz, gwilliams@svcc.biz, WCaddell@svcc.biz, gjackson@svcc.biz, mjackson@svcc.biz</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/3fmegrk2u3o7wws733ct6/ANSNJHoNIEr5TM8rxCTlWJw?rlkey=m7filqat6qhor7i9x1w8pqwqe&amp;st=kv7k3mv2&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2710,22 +2710,27 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Meals on Wheels</t>
+          <t>Men of Nehemiah</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/k1x3uhhsva3llk0r1vdxw/ADzOeKbPDUWS9rhgBWox-1M?rlkey=4u6z93o1v19wo5bqrdt62soig&amp;st=5q9fupd8&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/9mkztd08lp3l3r4a4tie9/AHCpk_Gb6xGUl5j3t53U_W4?rlkey=7ivp2llm5xtxqvomcq69nn4e5&amp;st=ou4zi9nh&amp;dl=0</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>cvargas@svcc.biz, kvirant@svcc.biz, gwilliams@svcc.biz, WCaddell@svcc.biz, gjackson@svcc.biz, mjackson@svcc.biz</t>
+          <t>cvargas@svcc.biz, jhenry@svcc.biz, wcaddell@svcc.biz, kregan@svcc.biz</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>https://app.procore.com/webclients/host/companies/29589/projects/2272839/tools/photos/albums/18343096?page=1&amp;sort=-exposure_date</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/3fmegrk2u3o7wws733ct6/ANSNJHoNIEr5TM8rxCTlWJw?rlkey=m7filqat6qhor7i9x1w8pqwqe&amp;st=kv7k3mv2&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/e14uuoltzhc3v19zmer3d/AH6F9clLql8-zhBpc4LR-4U?rlkey=vvxah7pv9fdmpcu62xsgmtwn5&amp;st=erfldgv5&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2737,27 +2742,27 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Men of Nehemiah</t>
+          <t>Northway Church Sanctuary</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/9mkztd08lp3l3r4a4tie9/AHCpk_Gb6xGUl5j3t53U_W4?rlkey=7ivp2llm5xtxqvomcq69nn4e5&amp;st=ou4zi9nh&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/a0uc9oixhjqf4e9mkwqgb/ACZCrvdACn1TpfpnrakaIeQ?rlkey=n2vh0kkd63b53ef1ga3brkafa&amp;st=04t2pc7v&amp;dl=0</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>cvargas@svcc.biz, jhenry@svcc.biz, wcaddell@svcc.biz, kregan@svcc.biz</t>
+          <t>mpage@svcc.biz, jpitrucha@svcc.biz, cmoore@svcc.biz, wcaddell@svcc.biz, cvargas@svcc.biz</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://app.procore.com/webclients/host/companies/29589/projects/2272839/tools/photos/albums/18343096?page=1&amp;sort=-exposure_date</t>
+          <t>https://app.procore.com/2749860/project/images/albums</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/e14uuoltzhc3v19zmer3d/AH6F9clLql8-zhBpc4LR-4U?rlkey=vvxah7pv9fdmpcu62xsgmtwn5&amp;st=erfldgv5&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/t7sz7fb813g5ac9lwj3cq/ALKLegkx90dN6Ujo5IxarHQ?rlkey=fdvmrx5hqcjmkv8fd4gmfkw96&amp;st=s9aj3r1n&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2769,27 +2774,27 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Northway Church Sanctuary</t>
+          <t>Silveron Park</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/a0uc9oixhjqf4e9mkwqgb/ACZCrvdACn1TpfpnrakaIeQ?rlkey=n2vh0kkd63b53ef1ga3brkafa&amp;st=04t2pc7v&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/pdto4ctrxxrbt3ui9xilb/AA4PMKE79OWn9pyN3AMhO6E?rlkey=i249og0mdaobt1dcmtkst43ed&amp;st=3n4nvn41&amp;dl=0</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>mpage@svcc.biz, jpitrucha@svcc.biz, cmoore@svcc.biz, wcaddell@svcc.biz, cvargas@svcc.biz</t>
+          <t>cvargas@svcc.biz, bhelm@svcc.biz, dmonk@svcc.biz, kregan@svcc.biz, wcaddell@svcc.biz</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>https://app.procore.com/2749860/project/images/albums</t>
+          <t>https://app.procore.com/2949565/project/images/show_album?id=18101370&amp;page=1&amp;sort=-exposure_date</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/t7sz7fb813g5ac9lwj3cq/ALKLegkx90dN6Ujo5IxarHQ?rlkey=fdvmrx5hqcjmkv8fd4gmfkw96&amp;st=s9aj3r1n&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/zwkaxbha7zdcbm2wh7tym/AJB4OMSEbICHSbdsFcUPQFA?rlkey=xoj2tie2ecijgjzj7z8zb5v7r&amp;st=yo1378be&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2801,27 +2806,27 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Silveron Park</t>
+          <t>The Bailey Rockwall</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/pdto4ctrxxrbt3ui9xilb/AA4PMKE79OWn9pyN3AMhO6E?rlkey=i249og0mdaobt1dcmtkst43ed&amp;st=3n4nvn41&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/nwsme6q5bjk1ako4nkswt/AM-3fIjsguE8DYExFN6LDJQ?rlkey=r0htpnlrrt0zmvwhtkjhdai9f&amp;st=zoz8w29y&amp;dl=0</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>cvargas@svcc.biz, bhelm@svcc.biz, dmonk@svcc.biz, kregan@svcc.biz, wcaddell@svcc.biz</t>
+          <t>cvargas@svcc.biz, Kpage@svcc.biz, wcaddell@svcc.biz, hmadison@svcc.biz</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>https://app.procore.com/2949565/project/images/show_album?id=18101370&amp;page=1&amp;sort=-exposure_date</t>
+          <t>https://app.procore.com/webclients/host/companies/29589/projects/1786527/tools/photos/albums</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/zwkaxbha7zdcbm2wh7tym/AJB4OMSEbICHSbdsFcUPQFA?rlkey=xoj2tie2ecijgjzj7z8zb5v7r&amp;st=yo1378be&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/ovys4x7brhsh822p6mnhu/AKbyGvZK66fav2BnQvSFKYg?rlkey=aeo6iv23yvbu913uru9d9163p&amp;st=1cy29ooo&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2833,27 +2838,27 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>The Bailey Rockwall</t>
+          <t>The Culbreath</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/nwsme6q5bjk1ako4nkswt/AM-3fIjsguE8DYExFN6LDJQ?rlkey=r0htpnlrrt0zmvwhtkjhdai9f&amp;st=zoz8w29y&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/bg1bvchczj2ju2qt547n6/ALQB2MrBYomFHuIgQTqJJjw?rlkey=000jhnb3gc6zodicfi7ugis1m&amp;st=j0n75da4&amp;dl=0</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>cvargas@svcc.biz, Kpage@svcc.biz, wcaddell@svcc.biz, hmadison@svcc.biz</t>
+          <t>cvargas@svcc.biz, rgartner@svcc.biz, bstahl@svcc.biz, mhernandez@svcc.biz, wcaddell@svcc.biz, Dana.Arnette@dhantx.com, dwelchel@voa.org</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://app.procore.com/webclients/host/companies/29589/projects/1786527/tools/photos/albums</t>
+          <t>https://app.procore.com/2824315/project/images/show_album?id=18068047&amp;page=1&amp;sort=-exposure_date</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/ovys4x7brhsh822p6mnhu/AKbyGvZK66fav2BnQvSFKYg?rlkey=aeo6iv23yvbu913uru9d9163p&amp;st=1cy29ooo&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/josep51wf5wrxz4bclibd/AHk1d1tkMwz0ktS939zDMZ8?rlkey=0gs2ft91vasv5kjq20gutt7g2&amp;st=1egh2tq3&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2865,59 +2870,54 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>The Culbreath</t>
+          <t>Tom Thumb Midlothian</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/bg1bvchczj2ju2qt547n6/ALQB2MrBYomFHuIgQTqJJjw?rlkey=000jhnb3gc6zodicfi7ugis1m&amp;st=j0n75da4&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/gnuv8q9apdlcf23hdtu0v/AMNIFkcEzgTQBzjv9N2JYXQ?rlkey=ot1k23w2ols5udd56pflvum2d&amp;st=xvg207ty&amp;dl=0</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>cvargas@svcc.biz, rgartner@svcc.biz, bstahl@svcc.biz, mhernandez@svcc.biz, wcaddell@svcc.biz, Dana.Arnette@dhantx.com, dwelchel@voa.org</t>
+          <t>cvargas@svcc.biz, mpage@svcc.biz, bwilson@svcc.biz, wcaddell@svcc.biz</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://app.procore.com/2824315/project/images/show_album?id=18068047&amp;page=1&amp;sort=-exposure_date</t>
+          <t>https://app.procore.com/webclients/host/companies/29589/projects/3066381/tools/photos/albums/18101347?page=1&amp;sort=-exposure_date</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/josep51wf5wrxz4bclibd/AHk1d1tkMwz0ktS939zDMZ8?rlkey=0gs2ft91vasv5kjq20gutt7g2&amp;st=1egh2tq3&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/gh0rz6thjcrwvbsx41lkt/AHpbbwIvn5NX8C_FMyJr6mw?rlkey=vzooihanqvldruemdrgl3nqzm&amp;st=s2tz4otl&amp;dl=0</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Spring Valley</t>
+          <t>Stillwater Capital</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Tom Thumb Midlothian</t>
+          <t>The Link Multifamily Phase 1</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/gnuv8q9apdlcf23hdtu0v/AMNIFkcEzgTQBzjv9N2JYXQ?rlkey=ot1k23w2ols5udd56pflvum2d&amp;st=xvg207ty&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/lhx9v67fm4wkvjc3ghjn4/ADJ7gQyLrxqNt5dXvF4Q49c?rlkey=0g7wagwxi7q4aqb3ggnlcz7zi&amp;st=hr1uj720&amp;dl=0</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>cvargas@svcc.biz, mpage@svcc.biz, bwilson@svcc.biz, wcaddell@svcc.biz</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>https://app.procore.com/webclients/host/companies/29589/projects/3066381/tools/photos/albums/18101347?page=1&amp;sort=-exposure_date</t>
+          <t>nathan.cordell@stillwatercapital.com, naomi.borrego@stillwatercap.com, alex.coval@stillwatercap.com, gary.green@stillwatercap.com, Steve.Garrison@StillwaterCapital.com, Jenny.Leporis@StillwaterCapital.com, Allen.LaSala@StillwaterCapital.com</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/gh0rz6thjcrwvbsx41lkt/AHpbbwIvn5NX8C_FMyJr6mw?rlkey=vzooihanqvldruemdrgl3nqzm&amp;st=s2tz4otl&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/esgnz3n19c0jo2uzc68g1/AGDqZI5PeoYXb_pY-0RqajY?rlkey=sbsd94jkml25igybxh26xp9vh&amp;st=u9014otj&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2929,49 +2929,49 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>The Link Multifamily Phase 1</t>
+          <t>Travis South</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/lhx9v67fm4wkvjc3ghjn4/ADJ7gQyLrxqNt5dXvF4Q49c?rlkey=0g7wagwxi7q4aqb3ggnlcz7zi&amp;st=hr1uj720&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/ohnsodr1xzm0x3x3nlaaw/AEcWPHIzbQbesbmHvIxRWIg?rlkey=y4t2p6dt64rbsyn2srx1gno0q&amp;st=7c03tzq2&amp;dl=0</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>nathan.cordell@stillwatercapital.com, naomi.borrego@stillwatercap.com, alex.coval@stillwatercap.com, gary.green@stillwatercap.com, Steve.Garrison@StillwaterCapital.com, Jenny.Leporis@StillwaterCapital.com, Allen.LaSala@StillwaterCapital.com</t>
+          <t>Steve.Garrison@StillwaterCapital.com, Landon.Wood@stillwatercap.com, jlenaerts@NHKCapitalPartners.com, mtemple@NHKCapitalPartners.com, nlee@cmbeb5visa.com, Allen.LaSala@StillwaterCapital.com, Sam.Hudson@StillwaterCapital.com</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/esgnz3n19c0jo2uzc68g1/AGDqZI5PeoYXb_pY-0RqajY?rlkey=sbsd94jkml25igybxh26xp9vh&amp;st=u9014otj&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/md4m0385w84yp2ix5c8a6/AArgEGF_0BayDcMGUQHdS3E?rlkey=41m5thnpp9g8vkvfgmby2zxgy&amp;st=fzmem3j3&amp;dl=0</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Stillwater Capital</t>
+          <t>Tellepsen</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Travis South</t>
+          <t>3425 W Alabama</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/ohnsodr1xzm0x3x3nlaaw/AEcWPHIzbQbesbmHvIxRWIg?rlkey=y4t2p6dt64rbsyn2srx1gno0q&amp;st=7c03tzq2&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/e3rrpxsu4kk62i3tz37eg/AAmeN4CLHUo9nF6TcpxWLP8?rlkey=3do5ujq5u1xxzjk14wr6zinzp&amp;st=v5htdwqc&amp;dl=0</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Steve.Garrison@StillwaterCapital.com, Landon.Wood@stillwatercap.com, jlenaerts@NHKCapitalPartners.com, mtemple@NHKCapitalPartners.com, nlee@cmbeb5visa.com, Allen.LaSala@StillwaterCapital.com, Sam.Hudson@StillwaterCapital.com</t>
+          <t>sbland@tellepsen.com, joffield@tellepsen.com, choward2@tellepsen.com</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/md4m0385w84yp2ix5c8a6/AArgEGF_0BayDcMGUQHdS3E?rlkey=41m5thnpp9g8vkvfgmby2zxgy&amp;st=fzmem3j3&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/b5m5jqsxxbme3plxusije/AMqqzf4Iep7mTJakif4TlaQ?rlkey=cxq9ljy2c6dw6b7yivxi9n829&amp;st=10zgvnch&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -2983,22 +2983,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>3425 W Alabama</t>
+          <t>Aldine MS</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/e3rrpxsu4kk62i3tz37eg/AAmeN4CLHUo9nF6TcpxWLP8?rlkey=3do5ujq5u1xxzjk14wr6zinzp&amp;st=v5htdwqc&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/dvf5ykddp37fmlwu3y7yf/ACKsilYmVDCJgK3blgWhapg?rlkey=vnrh5602t4wfdw3ku5buxbdow&amp;st=4q6vx088&amp;dl=0</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>sbland@tellepsen.com, joffield@tellepsen.com, choward2@tellepsen.com</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/b5m5jqsxxbme3plxusije/AMqqzf4Iep7mTJakif4TlaQ?rlkey=cxq9ljy2c6dw6b7yivxi9n829&amp;st=10zgvnch&amp;dl=0</t>
+          <t>Lhews@tellepsen.com, rwelch@tellepsen.com</t>
         </is>
       </c>
     </row>
@@ -3010,17 +3005,22 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Aldine MS</t>
+          <t>Camp For All</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/dvf5ykddp37fmlwu3y7yf/ACKsilYmVDCJgK3blgWhapg?rlkey=vnrh5602t4wfdw3ku5buxbdow&amp;st=4q6vx088&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/3owlu2d489gtp6sc4suhh/AMOwOiAqPr_5pY9gCVrS448?rlkey=fo0jhal8ivksxfok5kvpf3492&amp;st=d1i3o8om&amp;dl=0</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Lhews@tellepsen.com, rwelch@tellepsen.com</t>
+          <t>KMaerz@tellepsen.com, pperez@tellepsen.com, hescobar@tellepsen.com, cnelson@steadfastconstruction.us, ASlauson@tellepsen.com</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/gp6dzgg0ck207aumlzhzz/ABccL-MV9b7Aja9qJkQBJGE?rlkey=8qdg9o0kpuqzp4g7c2ysea8y7&amp;st=oo5xlbzr&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -3032,22 +3032,27 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Camp For All</t>
+          <t>CEE - Center for Jewish Leaning</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/3owlu2d489gtp6sc4suhh/AMOwOiAqPr_5pY9gCVrS448?rlkey=fo0jhal8ivksxfok5kvpf3492&amp;st=d1i3o8om&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/bgjh9wd6kq14ukkefn6rk/AC_SHeltX6_50X4HyEajPOI?rlkey=680vqu7d2wskawo48aunm2ppi&amp;st=9ffnahub&amp;dl=0</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>KMaerz@tellepsen.com, pperez@tellepsen.com, hescobar@tellepsen.com, cnelson@steadfastconstruction.us, ASlauson@tellepsen.com</t>
+          <t>dcontreras@tellepsen.com, BCooper@tellepsen.com, hescobar@tellepsen.com</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>https://us02.procore.com/562949954549392/project/images/show_album?id=562949958635784&amp;page=1&amp;sort=-exposure_date</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/gp6dzgg0ck207aumlzhzz/ABccL-MV9b7Aja9qJkQBJGE?rlkey=8qdg9o0kpuqzp4g7c2ysea8y7&amp;st=oo5xlbzr&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/9c7golo8puf8mb1zxxdtf/AM6M3wNoH-l1ei7shRtZIPc?rlkey=kppej3kix70a1rkhuq0yg0xf4&amp;st=9kyhs4pq&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -3059,27 +3064,22 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>CEE - Center for Jewish Leaning</t>
+          <t>HCU Building</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/bgjh9wd6kq14ukkefn6rk/AC_SHeltX6_50X4HyEajPOI?rlkey=680vqu7d2wskawo48aunm2ppi&amp;st=9ffnahub&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/528pvm6omdmyzzt2xaw6o/ADDWE-fwLj4NJ_snjatIRHA?rlkey=1jolnftw93siyds9nrp20ufr7&amp;st=r82i4itr&amp;dl=0</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>dcontreras@tellepsen.com, BCooper@tellepsen.com, hescobar@tellepsen.com</t>
+          <t>CLaPlant@tellepsen.com, SFlores@tellepsen.com, TSchoener@tellepsen.com, ZZamora@tellepsen.com</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>https://us02.procore.com/562949954549392/project/images/show_album?id=562949958635784&amp;page=1&amp;sort=-exposure_date</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/9c7golo8puf8mb1zxxdtf/AM6M3wNoH-l1ei7shRtZIPc?rlkey=kppej3kix70a1rkhuq0yg0xf4&amp;st=9kyhs4pq&amp;dl=0</t>
+          <t>https://us02.procore.com/562949954755274/project/images/show_album?id=562949958641018&amp;page=1&amp;sort=-exposure_date</t>
         </is>
       </c>
     </row>
@@ -3091,22 +3091,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>HCU Building</t>
+          <t>Hempstead HS</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/528pvm6omdmyzzt2xaw6o/ADDWE-fwLj4NJ_snjatIRHA?rlkey=1jolnftw93siyds9nrp20ufr7&amp;st=r82i4itr&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/x3omcqoxeatdpbhllc46a/ACX85SDI2wcz5r9MR-2zSsQ?rlkey=o4ue0zfxai76q03pj9jhe57yx&amp;st=llwz4dv7&amp;dl=0</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>CLaPlant@tellepsen.com, SFlores@tellepsen.com, TSchoener@tellepsen.com, ZZamora@tellepsen.com</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>https://us02.procore.com/562949954755274/project/images/show_album?id=562949958641018&amp;page=1&amp;sort=-exposure_date</t>
+          <t>Afulton@tellepsen.com</t>
         </is>
       </c>
     </row>
@@ -3118,17 +3113,22 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Hempstead HS</t>
+          <t>Hempstead ISD - Early Childhood Center Project</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/x3omcqoxeatdpbhllc46a/ACX85SDI2wcz5r9MR-2zSsQ?rlkey=o4ue0zfxai76q03pj9jhe57yx&amp;st=llwz4dv7&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/xvdxjqlwajji2vobiqizx/AAq9QUqSv3ncm5RuRLEfyxs?rlkey=a3m8u1fow6b57dhhqmxowa6f0&amp;st=vbp4bhy8&amp;dl=0</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Afulton@tellepsen.com</t>
+          <t>afulton@tellepsen.com</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/tw10e6vkjcrrneoz3i3uz/AG1uC5yrhVya8-z9ev8-N0M?rlkey=fnxh0umk5y3d5fj3a0i296ja3&amp;st=n9hi14eg&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -3140,22 +3140,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Hempstead ISD - Early Childhood Center Project</t>
+          <t>Hempstead MS</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/xvdxjqlwajji2vobiqizx/AAq9QUqSv3ncm5RuRLEfyxs?rlkey=a3m8u1fow6b57dhhqmxowa6f0&amp;st=vbp4bhy8&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/oxs4c1cb5rej8vfo5jqut/AM7cxTX1z8rvTLvCSpjCKak?rlkey=0b0n3yllzuac9718n4noxa9uc&amp;st=dym9sxyk&amp;dl=0</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>afulton@tellepsen.com</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/tw10e6vkjcrrneoz3i3uz/AG1uC5yrhVya8-z9ev8-N0M?rlkey=fnxh0umk5y3d5fj3a0i296ja3&amp;st=n9hi14eg&amp;dl=0</t>
+          <t>Afulton@tellepsen.com</t>
         </is>
       </c>
     </row>
@@ -3167,17 +3162,27 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Hempstead MS</t>
+          <t xml:space="preserve">LBJ CUP </t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/oxs4c1cb5rej8vfo5jqut/AM7cxTX1z8rvTLvCSpjCKak?rlkey=0b0n3yllzuac9718n4noxa9uc&amp;st=dym9sxyk&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/4rsjv9halofzr36cj02ll/AGrDmqhjHMDhkG90AT4-Nwo?rlkey=v1lg644c7y7gnv7pwrckznvf5&amp;st=0ey42270&amp;dl=0</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Afulton@tellepsen.com</t>
+          <t>zmoffitt@tellepsen.com, nherzinger@tellepsen.com, JHoesel@tellepsen.com</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>https://us02.procore.com/562949954659712/project/images/albums</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/wj1852zv6w0p27fop9jov/ADXhrXfoCtMPBV5mxdmerOA?rlkey=xm6sokwy8o3j10ty6k2m7xwfe&amp;st=pc1iely3&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -3189,27 +3194,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">LBJ CUP </t>
+          <t>Lifetime Harvest Green</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/4rsjv9halofzr36cj02ll/AGrDmqhjHMDhkG90AT4-Nwo?rlkey=v1lg644c7y7gnv7pwrckznvf5&amp;st=0ey42270&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/v01m98muqx46wjtle90bn/AD-wGMCwd8LhRoQk0xoeGqo?rlkey=fwi3y9l632pj0ngd8mm4ie2z8&amp;st=cnpt99gx&amp;dl=0</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>zmoffitt@tellepsen.com, nherzinger@tellepsen.com, JHoesel@tellepsen.com</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>https://us02.procore.com/562949954659712/project/images/albums</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/wj1852zv6w0p27fop9jov/ADXhrXfoCtMPBV5mxdmerOA?rlkey=xm6sokwy8o3j10ty6k2m7xwfe&amp;st=pc1iely3&amp;dl=0</t>
+          <t>CTaylor@tellepsen.com</t>
         </is>
       </c>
     </row>
@@ -3221,17 +3216,27 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Lifetime Harvest Green</t>
+          <t>McCullough ISD</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/v01m98muqx46wjtle90bn/AD-wGMCwd8LhRoQk0xoeGqo?rlkey=fwi3y9l632pj0ngd8mm4ie2z8&amp;st=cnpt99gx&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/1m911gpphs60r0ts2796e/ANfLjUMiz87lNynqr3EmiNM?rlkey=vhhbl1z2165h9rjfrqmxbljhp&amp;st=uhsfgveb&amp;dl=0</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>CTaylor@tellepsen.com</t>
+          <t>TWilliams2@tellepsen.com</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>https://us02.procore.com/webclients/host/companies/562949953505905/projects/562949954694811/tools/photos/albums/562949959298566?page=1&amp;sort=-exposure_date</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/pdafe9elyc1m8wn4rxakf/AIk2J6el0EGbRUmT1RRb2eQ?rlkey=nutdzhbsqwfqmmmehwc7l3me9&amp;st=n8a87egp&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -3243,27 +3248,22 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>McCullough ISD</t>
+          <t>Memorial Hermann Sugar Land</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/1m911gpphs60r0ts2796e/ANfLjUMiz87lNynqr3EmiNM?rlkey=vhhbl1z2165h9rjfrqmxbljhp&amp;st=uhsfgveb&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/hrdvvcy3wkmamac4txz8y/AFvxhcCFKf4KwgphonNkDt4?rlkey=0p8dlwujmn45qc6kkmivh79po&amp;st=0wd8wskq&amp;dl=0</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>TWilliams2@tellepsen.com</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>https://us02.procore.com/webclients/host/companies/562949953505905/projects/562949954694811/tools/photos/albums/562949959298566?page=1&amp;sort=-exposure_date</t>
+          <t>drauch@tellepsen.com, rzeutschel@tellepsen.com, gkubecka@tellepsen.com</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/pdafe9elyc1m8wn4rxakf/AIk2J6el0EGbRUmT1RRb2eQ?rlkey=nutdzhbsqwfqmmmehwc7l3me9&amp;st=n8a87egp&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/rkj13whab48n69s7bvqsx/ADU8U5lb3WQOrz3UgTXdPfU?rlkey=x4pqccwppcnlqh91gqwwl0d6g&amp;st=8j7pt7ll&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -3275,22 +3275,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Memorial Hermann Sugar Land</t>
+          <t>Memorial Park Groves</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/hrdvvcy3wkmamac4txz8y/AFvxhcCFKf4KwgphonNkDt4?rlkey=0p8dlwujmn45qc6kkmivh79po&amp;st=0wd8wskq&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/y6oh1ib7k34q5ulxk1iur/AK1ICdg6r_CGUMw2-Ogqr2k?rlkey=neboe4nyam8dkjj8fwb9pokru&amp;st=rlr6mwz5&amp;dl=0</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>drauch@tellepsen.com, rzeutschel@tellepsen.com, gkubecka@tellepsen.com</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/rkj13whab48n69s7bvqsx/ADU8U5lb3WQOrz3UgTXdPfU?rlkey=x4pqccwppcnlqh91gqwwl0d6g&amp;st=8j7pt7ll&amp;dl=0</t>
+          <t>Ekolupski@tellepsen.com, MAndaya@tellepsen.com</t>
         </is>
       </c>
     </row>
@@ -3302,17 +3297,22 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Memorial Park Groves</t>
+          <t>South Bank Trail</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/y6oh1ib7k34q5ulxk1iur/AK1ICdg6r_CGUMw2-Ogqr2k?rlkey=neboe4nyam8dkjj8fwb9pokru&amp;st=rlr6mwz5&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/9n0cz0usae1fy4dchcmo6/AIRDaoGcytu0uEknY5_hOD0?rlkey=cc4mxszbyav26k6phjow1piur&amp;st=bbj4js1f&amp;dl=0</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Ekolupski@tellepsen.com, MAndaya@tellepsen.com</t>
+          <t>djuarez@tellepsen.com, dmckee@tellepsen.com</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/hjfikv9gujmw6lyd4bguc/AGrB3fDqcLG8gtrFJTXNfxw?rlkey=q05y7prky43y3wq7gek3vcfed&amp;st=9dbuq9i9&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -3324,22 +3324,27 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>South Bank Trail</t>
+          <t>Tony Marron Park East</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/9n0cz0usae1fy4dchcmo6/AIRDaoGcytu0uEknY5_hOD0?rlkey=cc4mxszbyav26k6phjow1piur&amp;st=bbj4js1f&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/7z2f7ya19ea2na8vpp6tu/ANctFcpfwAE779b70yrCSXM?rlkey=qp5eezwarm0f99ismfvyzuoki&amp;st=gqi3p98d&amp;dl=0</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>djuarez@tellepsen.com, dmckee@tellepsen.com</t>
+          <t>cmcpherson@tellepsen.com</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>https://us02.procore.com/562949954275515/project/images/show_album?id=562949958235457&amp;page=1&amp;sort=-exposure_date</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/hjfikv9gujmw6lyd4bguc/AGrB3fDqcLG8gtrFJTXNfxw?rlkey=q05y7prky43y3wq7gek3vcfed&amp;st=9dbuq9i9&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/69pd51cbajm5tja7a6wg4/AMPgUDGXj4BaKoqgoMJY_3o?rlkey=1y5ol9v2kky5xoimzcn6t5kwb&amp;st=hiov94la&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -3351,108 +3356,98 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Tony Marron Park East</t>
+          <t>Tony Marron Park West</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/7z2f7ya19ea2na8vpp6tu/ANctFcpfwAE779b70yrCSXM?rlkey=qp5eezwarm0f99ismfvyzuoki&amp;st=gqi3p98d&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/v8yjp40pw6azgn87u956n/AFLMg3sPuynqEul5vS8mGp0?rlkey=5xmaowirxg8gww2tmey5sej9e&amp;st=ve34qua8&amp;dl=0</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>cmcpherson@tellepsen.com</t>
+          <t>cmcpherson@tellepsen.com, rarredondo@tellepsen.com</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>https://us02.procore.com/562949954275515/project/images/show_album?id=562949958235457&amp;page=1&amp;sort=-exposure_date</t>
+          <t>https://us02.procore.com/562949954275515/project/images/show_album?id=562949957654337&amp;page=1&amp;sort=-exposure_date</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/69pd51cbajm5tja7a6wg4/AMPgUDGXj4BaKoqgoMJY_3o?rlkey=1y5ol9v2kky5xoimzcn6t5kwb&amp;st=hiov94la&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/jo6bq21kh8wgtsjjrbomv/AC0TbIJrV-j-ML4RGv-dTZY?rlkey=4737wsvszo8xh4kfkvz23tzea&amp;st=o6u5w1hj&amp;dl=0</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Tellepsen</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Tony Marron Park West</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/v8yjp40pw6azgn87u956n/AFLMg3sPuynqEul5vS8mGp0?rlkey=5xmaowirxg8gww2tmey5sej9e&amp;st=ve34qua8&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/2u22rkfy8auzr19nq103s/AKCiHNTg1Lei6w9LW-Rrq0k?rlkey=bnrbpwsdjrb740q2tnlc3w34y&amp;st=bwn17cis&amp;dl=0</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>cmcpherson@tellepsen.com, rarredondo@tellepsen.com</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>https://us02.procore.com/562949954275515/project/images/show_album?id=562949957654337&amp;page=1&amp;sort=-exposure_date</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/jo6bq21kh8wgtsjjrbomv/AC0TbIJrV-j-ML4RGv-dTZY?rlkey=4737wsvszo8xh4kfkvz23tzea&amp;st=o6u5w1hj&amp;dl=0</t>
+          <t>smclaren@archaerial.com</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>TEST</t>
+          <t>TriArc</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>TEST</t>
+          <t>ICI Oasis Mixed Use</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/2u22rkfy8auzr19nq103s/AKCiHNTg1Lei6w9LW-Rrq0k?rlkey=bnrbpwsdjrb740q2tnlc3w34y&amp;st=bwn17cis&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/w34i30vmep2v7rb5f3zm8/ANhJT_A92bujPXjQQBeLhYI?rlkey=597gdzbpttcm4bavrns5kcu0k&amp;st=b0dhv9kt&amp;dl=0</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>smclaren@archaerial.com</t>
+          <t>shane@triarc-llc.com, amunoz@triarc-llc.com, jthompson@triarc-llc.com</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/7gifomyhm1ksa1s9ouk88/AOzX38yoVaNyMIs5I9DQXpw?rlkey=poluupb1ajhiceuqh498k2mdw&amp;st=p8lg0w56&amp;dl=0</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>TriArc</t>
+          <t>Weber &amp; Company</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>ICI Oasis Mixed Use</t>
+          <t>Epic West Towne Crossing</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/w34i30vmep2v7rb5f3zm8/ANhJT_A92bujPXjQQBeLhYI?rlkey=597gdzbpttcm4bavrns5kcu0k&amp;st=b0dhv9kt&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/e7qqlh7hna7p1wjnp23tq/AIMtqAUq5n5_wqX_C2LIDZI?rlkey=z9x2n78xxlbyvevrqp5664f0f&amp;st=yonqab1t&amp;dl=0</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>shane@triarc-llc.com, amunoz@triarc-llc.com, jthompson@triarc-llc.com</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/7gifomyhm1ksa1s9ouk88/AOzX38yoVaNyMIs5I9DQXpw?rlkey=poluupb1ajhiceuqh498k2mdw&amp;st=p8lg0w56&amp;dl=0</t>
+          <t>michael.davis@weberandcompany.com</t>
         </is>
       </c>
     </row>
@@ -3464,12 +3459,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Epic West Towne Crossing</t>
+          <t>Target Little Elm</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/e7qqlh7hna7p1wjnp23tq/AIMtqAUq5n5_wqX_C2LIDZI?rlkey=z9x2n78xxlbyvevrqp5664f0f&amp;st=yonqab1t&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/atcx0duon06euutxgf6uz/ADl33Sk3YcSnoL5apGqK8ko?rlkey=6qbrmey34k4yqptv4vpn53isc&amp;st=671mi5qh&amp;dl=0</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3481,22 +3476,27 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Weber &amp; Company</t>
+          <t>Z Constructors</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Target Little Elm</t>
+          <t>Auto Park Dallas</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/atcx0duon06euutxgf6uz/ADl33Sk3YcSnoL5apGqK8ko?rlkey=6qbrmey34k4yqptv4vpn53isc&amp;st=671mi5qh&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/hc5d0ky6qbgspofbonhuh/AGYaHMGsFj28vK4I9JW_gYw?rlkey=njykoxd52clgz3mvcluhic8b7&amp;st=swwsax4n&amp;dl=0</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>michael.davis@weberandcompany.com</t>
+          <t>mmccarter@zconstructors.com, tgeorge@zconstructors.com, cbowles@zconstructors.com, JLeckie@zconstructors.com, BGoodman@zconstructors.com</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/vqgwqz9g228lr4br4yala/AGL_aZX4rP245k4dbn8qxG4?rlkey=n9egqyvkzhlu1wmxg4w44djth&amp;st=m4gdiiw0&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -3508,22 +3508,22 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Auto Park Dallas</t>
+          <t>HG Supply Co</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/hc5d0ky6qbgspofbonhuh/AGYaHMGsFj28vK4I9JW_gYw?rlkey=njykoxd52clgz3mvcluhic8b7&amp;st=swwsax4n&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/2jneqj2ineo6rao3wlbgc/ALfEbccOU-r25SSqGpG-Ee0?rlkey=34gdlm0h577b5auv079zwap7k&amp;st=f8vdhybi&amp;dl=0</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>mmccarter@zconstructors.com, tgeorge@zconstructors.com, cbowles@zconstructors.com, JLeckie@zconstructors.com, BGoodman@zconstructors.com</t>
+          <t>cwest@zconstructors.com, JLeckie@zconstructors.com, jlanier@zconstructors.com, smcgaha@zconstructors.com</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/vqgwqz9g228lr4br4yala/AGL_aZX4rP245k4dbn8qxG4?rlkey=n9egqyvkzhlu1wmxg4w44djth&amp;st=m4gdiiw0&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/8ztwa7c68zh1r0gdbjhwf/AGTjh6rbEI-_Q08I6QR5gyE?rlkey=skjv69ty37twt2du1n4gwjbyh&amp;st=b9myo9xz&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -3535,22 +3535,22 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>HG Supply Co</t>
+          <t>Quality Collision The Colony</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/2jneqj2ineo6rao3wlbgc/ALfEbccOU-r25SSqGpG-Ee0?rlkey=34gdlm0h577b5auv079zwap7k&amp;st=f8vdhybi&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/ec52f6ln5fznmlv6g2vot/AG49CtbntZ9XYgpF896wf20?rlkey=slbs0se42ejrlkoyvh5vj7tif&amp;st=ipbxcfkb&amp;dl=0</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>cwest@zconstructors.com, JLeckie@zconstructors.com, jlanier@zconstructors.com, smcgaha@zconstructors.com</t>
+          <t>cwest@zconstructors.com, JLeckie@zconstructors.com, smcgaha@zconstructors.com, jherron@zconstructors.com</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/8ztwa7c68zh1r0gdbjhwf/AGTjh6rbEI-_Q08I6QR5gyE?rlkey=skjv69ty37twt2du1n4gwjbyh&amp;st=b9myo9xz&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/yu0qb276jo98zvsl3bmkb/AHBxjozSxKtMmdWez7LvqOY?rlkey=w8z5y2f7u4j5x7mcb4a3vfd24&amp;st=bx0s1e0e&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -3562,47 +3562,20 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Quality Collision The Colony</t>
+          <t>The Hub of Rowlett</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/ec52f6ln5fznmlv6g2vot/AG49CtbntZ9XYgpF896wf20?rlkey=slbs0se42ejrlkoyvh5vj7tif&amp;st=ipbxcfkb&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/fw05xwmsrzilkxvt83egu/AFl_XVDCw9aaCluq12G2Ky8?rlkey=0u77hgrf9kv7y392y7e4rmckb&amp;st=kftl8yme&amp;dl=0</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>cwest@zconstructors.com, JLeckie@zconstructors.com, smcgaha@zconstructors.com, jherron@zconstructors.com</t>
+          <t>cwest@zconstructors.com, jlanier@zconstructors.com, JLeckie@zconstructors.com, smcgaha@zconstructors.com</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/yu0qb276jo98zvsl3bmkb/AHBxjozSxKtMmdWez7LvqOY?rlkey=w8z5y2f7u4j5x7mcb4a3vfd24&amp;st=bx0s1e0e&amp;dl=0</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>Z Constructors</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>The Hub of Rowlett</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/fw05xwmsrzilkxvt83egu/AFl_XVDCw9aaCluq12G2Ky8?rlkey=0u77hgrf9kv7y392y7e4rmckb&amp;st=kftl8yme&amp;dl=0</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>cwest@zconstructors.com, jlanier@zconstructors.com, JLeckie@zconstructors.com, smcgaha@zconstructors.com</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
         <is>
           <t>https://www.dropbox.com/scl/fo/z5jwz4ybcq739vhtb8aan/AJb341FJ9ejf9y5Htk-Rmd4?rlkey=cc2kavhs09vbzg04tcyofngfj&amp;st=rs5vb3t2&amp;dl=0</t>
         </is>
@@ -4271,7 +4244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35.5703125" customWidth="1" min="1" max="2"/>
@@ -4836,22 +4809,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Schwob</t>
+          <t>Satterfield &amp; Pontikes</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Estes Express Lines</t>
+          <t>Chambers County Justice Center</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/rcxfcmvkgqhw7d9u09oe4/ALjyzjGyXjZdEulLRKJtyxM?rlkey=qpg0lxcwef7dx2gyol52v2z7w&amp;st=m3yx0ay3&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/9yksjubv94yr5wbu1f80t/APweuR7mw621WYxZ-8rBWR0?rlkey=l2wjt0a9alatgmnacnkj03j9k&amp;st=hzt8gnf3&amp;dl=0</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>abattard@schwob.com, eknott@schwob.com</t>
+          <t>bchobot@satpon.com, jcervantes@satpon.com, dbihn@satpon.com, mrasmussen@satpon.com, aguerrero@satpon.com, pball@satpon.com, jshepherd@satpon.com, tgranato@satpon.com</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/19ja32kmfghcbjxrgzpco/AEMXdgEtC985yTE-xR25oK8?rlkey=r2iz880hojxs7kdoz1xjnmg72&amp;st=o3nxotzq&amp;dl=0</t>
         </is>
       </c>
     </row>
@@ -4863,17 +4841,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ODFL Corpus</t>
+          <t>Estes Express Lines</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/87yo8cwod3pf88vdumxyn/APST7AEi9c4DBukwyK0IchE?rlkey=ayvjp4zsqppdc6mjbq1778hpc&amp;st=5dxr5diq&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/rcxfcmvkgqhw7d9u09oe4/ALjyzjGyXjZdEulLRKJtyxM?rlkey=qpg0lxcwef7dx2gyol52v2z7w&amp;st=m3yx0ay3&amp;dl=0</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>erush@schwob.com, mdavenport@schwob.com, jalford@schwob.com, sbyard@schwob.com</t>
+          <t>abattard@schwob.com, eknott@schwob.com</t>
         </is>
       </c>
     </row>
@@ -4885,17 +4863,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SAIA Dock Expansion</t>
+          <t>ODFL Corpus</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/1uukfwd68s0mofiv11h6n/AOL8660hZneA8jkNgM4RNDQ?rlkey=6n2h7ub4c763l0j52t9v0g8dy&amp;st=7eyadyxj&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/87yo8cwod3pf88vdumxyn/APST7AEi9c4DBukwyK0IchE?rlkey=ayvjp4zsqppdc6mjbq1778hpc&amp;st=5dxr5diq&amp;dl=0</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>eknott@schwob.com, jmaxton@schwob.com</t>
+          <t>erush@schwob.com, mdavenport@schwob.com, jalford@schwob.com, sbyard@schwob.com</t>
         </is>
       </c>
     </row>
@@ -4907,66 +4885,61 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SEFL Houston</t>
+          <t>SAIA Dock Expansion</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/57d9958hjut7qwzevpsfz/AM2TvUKKne372kp41v7eBjY?rlkey=j53euqg9e23tnevsjubnsoeg0&amp;st=l10au04t&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/1uukfwd68s0mofiv11h6n/AOL8660hZneA8jkNgM4RNDQ?rlkey=6n2h7ub4c763l0j52t9v0g8dy&amp;st=7eyadyxj&amp;dl=0</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>rkorthauer@schwob.com, rsnyder@schwob.com</t>
+          <t>eknott@schwob.com, jmaxton@schwob.com</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SpawGlass</t>
+          <t>Schwob</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>100 E Methvin St</t>
+          <t>SEFL Houston</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/ouwmo2qdujm0nv8pvokqy/ANei0rTs2KqqHjKxgKS3uio?rlkey=e2whiplov80fp1ayb7oh2w9wp&amp;st=e586zgpq&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/57d9958hjut7qwzevpsfz/AM2TvUKKne372kp41v7eBjY?rlkey=j53euqg9e23tnevsjubnsoeg0&amp;st=l10au04t&amp;dl=0</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>connor.cook@spawglass.om, drake.jolley@spawglass.com, brett.fast@spawglass.com, landon.floyd@spawglass.com</t>
+          <t>rkorthauer@schwob.com, rsnyder@schwob.com</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Spring Valley</t>
+          <t>SpawGlass</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Gateway Park</t>
+          <t>100 E Methvin St</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/hlrkju0rznqajmxdbkpck/AGISH036wXbEXvnwJBBfvfY?rlkey=qxrqg4ax4mp8y50jpxop2ps3r&amp;st=gtk18nwq&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/ouwmo2qdujm0nv8pvokqy/ANei0rTs2KqqHjKxgKS3uio?rlkey=e2whiplov80fp1ayb7oh2w9wp&amp;st=e586zgpq&amp;dl=0</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>kpage@svcc.biz, wcaddell@svcc.biz, cvargas@svcc.biz</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>https://app.procore.com/webclients/host/companies/29589/projects/2918239/tools/photos/albums</t>
+          <t>connor.cook@spawglass.om, drake.jolley@spawglass.com, brett.fast@spawglass.com, landon.floyd@spawglass.com</t>
         </is>
       </c>
     </row>
@@ -4978,22 +4951,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>IKEA Phase 2</t>
+          <t>Gateway Park</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/7l2reez6j329llg5y2ppy/AOdktsxwDcF3w9e3aM4ryU0?rlkey=e09agth3k7l2hqxpb77tbdehc&amp;st=nletvul6&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/hlrkju0rznqajmxdbkpck/AGISH036wXbEXvnwJBBfvfY?rlkey=qxrqg4ax4mp8y50jpxop2ps3r&amp;st=gtk18nwq&amp;dl=0</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>cvargas@svcc.biz, mpage@svcc.biz, mwarwick@svcc.biz, klong@svcc.biz, wcaddell@svcc.biz</t>
+          <t>kpage@svcc.biz, wcaddell@svcc.biz, cvargas@svcc.biz</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://app.procore.com/2999366/project/images/albums</t>
+          <t>https://app.procore.com/webclients/host/companies/29589/projects/2918239/tools/photos/albums</t>
         </is>
       </c>
     </row>
@@ -5005,22 +4978,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Main Street Towne Crossing Midlothian</t>
+          <t>IKEA Phase 2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/muj7kx4uvxgs0ewze64r4/AFSD0Dpa8EWk7xYa0svIhfs?rlkey=2f6ywl8e3u07ge4gm41y122am&amp;st=t4v469yy&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/7l2reez6j329llg5y2ppy/AOdktsxwDcF3w9e3aM4ryU0?rlkey=e09agth3k7l2hqxpb77tbdehc&amp;st=nletvul6&amp;dl=0</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>cvargas@svcc.biz, ccarlisle@svcc.biz, kvirant@svcc.biz, cmoore@svcc.biz, wcaddell@svcc.biz</t>
+          <t>cvargas@svcc.biz, mpage@svcc.biz, mwarwick@svcc.biz, klong@svcc.biz, wcaddell@svcc.biz</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://app.procore.com/webclients/host/companies/29589/projects/2800907/tools/photos/albums</t>
+          <t>https://app.procore.com/2999366/project/images/albums</t>
         </is>
       </c>
     </row>
@@ -5032,49 +5005,49 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>The Stream at High Pointe</t>
+          <t>Main Street Towne Crossing Midlothian</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/sslxae1hzpqve2vsyqh7s/ALkIQrZU_slG85bMj5Xax3k?rlkey=jhr65yw6hx3hui62ijdwdc8us&amp;st=e7rcpbj5&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/muj7kx4uvxgs0ewze64r4/AFSD0Dpa8EWk7xYa0svIhfs?rlkey=2f6ywl8e3u07ge4gm41y122am&amp;st=t4v469yy&amp;dl=0</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>cvargas@svcc.biz, sgross@svcc.biz, cstringer@svcc.biz, hbrittain@svcc.biz, wcaddell@svcc.biz</t>
+          <t>cvargas@svcc.biz, ccarlisle@svcc.biz, kvirant@svcc.biz, cmoore@svcc.biz, wcaddell@svcc.biz</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://app.procore.com/2012586/project/images/albums</t>
+          <t>https://app.procore.com/webclients/host/companies/29589/projects/2800907/tools/photos/albums</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Tellepsen</t>
+          <t>Spring Valley</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Lockwood Park</t>
+          <t>The Stream at High Pointe</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/ral09t2euw7qdof1wqnyl/AHWUWp3MdYXPvduX5VSDG-0?rlkey=vad5iqr1qa89aghj82da01nfd&amp;st=gn7hm84b&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/sslxae1hzpqve2vsyqh7s/ALkIQrZU_slG85bMj5Xax3k?rlkey=jhr65yw6hx3hui62ijdwdc8us&amp;st=e7rcpbj5&amp;dl=0</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>djuarez@tellepsen.com</t>
+          <t>cvargas@svcc.biz, sgross@svcc.biz, cstringer@svcc.biz, hbrittain@svcc.biz, wcaddell@svcc.biz</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://us02.procore.com/562949954304914/project/images/albums</t>
+          <t>https://app.procore.com/2012586/project/images/albums</t>
         </is>
       </c>
     </row>
@@ -5086,22 +5059,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lomax Jr High </t>
+          <t>Lockwood Park</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/5sqof6dfspxklbrdfk5x0/AO6eUnB8gSkOuE7NnE4joCU?rlkey=slqds8ui42ddp4uel407bkilp&amp;st=cljg6hzn&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/ral09t2euw7qdof1wqnyl/AHWUWp3MdYXPvduX5VSDG-0?rlkey=vad5iqr1qa89aghj82da01nfd&amp;st=gn7hm84b&amp;dl=0</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>ARoberts@tellepsen.com, hlarkin@tellepsen.com, jcoffee@tellepsen.com, cshanley@tellepsen.com</t>
+          <t>djuarez@tellepsen.com</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://us02.procore.com/562949954668752/project/images/albums</t>
+          <t>https://us02.procore.com/562949954304914/project/images/albums</t>
         </is>
       </c>
     </row>
@@ -5113,61 +5086,66 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Sweeny Community Hospital</t>
+          <t xml:space="preserve">Lomax Jr High </t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/fvdhew4g8gs3i3eyrtx7p/AKTqn60HxuGx_-TrPfUwXiQ?rlkey=qjwrl2u1g14rt5o1phk81grn1&amp;st=a7wocmnx&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/5sqof6dfspxklbrdfk5x0/AO6eUnB8gSkOuE7NnE4joCU?rlkey=slqds8ui42ddp4uel407bkilp&amp;st=cljg6hzn&amp;dl=0</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>lmurphy@tellepsen.com, zzamora@tellepsen.com, jcoots@tellepsen.com</t>
+          <t>ARoberts@tellepsen.com, hlarkin@tellepsen.com, jcoffee@tellepsen.com, cshanley@tellepsen.com</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://us02.procore.com/562949954668752/project/images/albums</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TriArc</t>
+          <t>Tellepsen</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Anjuman School</t>
+          <t>Sweeny Community Hospital</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/tqmn3vh5ei68dkz1p3e85/AONY3qOO9BnBIp6irmbstQQ?rlkey=5q95ie7g611jtlhxdywe91iox&amp;st=qsqrk8qk&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/fvdhew4g8gs3i3eyrtx7p/AKTqn60HxuGx_-TrPfUwXiQ?rlkey=qjwrl2u1g14rt5o1phk81grn1&amp;st=a7wocmnx&amp;dl=0</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>shane@triarc-llc.com, amunoz@triarc-llc.com, macyfaithking@gmail.com</t>
+          <t>lmurphy@tellepsen.com, zzamora@tellepsen.com, jcoots@tellepsen.com</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Z Constructors</t>
+          <t>TriArc</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Lowe Tractor Dealership</t>
+          <t>Anjuman School</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/fiyw8k18de2qtn2iz8qzz/AM3As2ii9Wjs3sqsNZ4d4y0?rlkey=z7cmn9ricob2mzxjl6w6kgq27&amp;st=hu8ngzc3&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/tqmn3vh5ei68dkz1p3e85/AONY3qOO9BnBIp6irmbstQQ?rlkey=5q95ie7g611jtlhxdywe91iox&amp;st=qsqrk8qk&amp;dl=0</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Mwiskur@zconstructors.com, Cfloyd@zconstructors.com, JLeckie@zconstructors.com, jherron@zconstructors.com</t>
+          <t>shane@triarc-llc.com, amunoz@triarc-llc.com, macyfaithking@gmail.com</t>
         </is>
       </c>
     </row>
@@ -5179,15 +5157,37 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>Lowe Tractor Dealership</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/fiyw8k18de2qtn2iz8qzz/AM3As2ii9Wjs3sqsNZ4d4y0?rlkey=z7cmn9ricob2mzxjl6w6kgq27&amp;st=hu8ngzc3&amp;dl=0</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Mwiskur@zconstructors.com, Cfloyd@zconstructors.com, JLeckie@zconstructors.com, jherron@zconstructors.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Z Constructors</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>Quality Collision Fort Worth</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>https://www.dropbox.com/scl/fo/2u8zrjnonyi8ygmxv7mt9/AOEkPaYWXz8mWV-YBqyGXOQ?rlkey=mw1wcqb54u4uvo0npnx909n94&amp;st=2fds3bt3&amp;dl=0</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>cwest@zconstructors.com, tdossett@zconstructors.com, JLeckie@zconstructors.com</t>
         </is>

</xml_diff>

<commit_message>
Reverted adjustments made for Outlook (Not Classic) | Updated Customer Info
</commit_message>
<xml_diff>
--- a/Reference Data/XLSX Workbooks/Customer Information.xlsx
+++ b/Reference Data/XLSX Workbooks/Customer Information.xlsx
@@ -3630,7 +3630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78.42578125" customWidth="1" min="1" max="2"/>
@@ -3666,6 +3666,15 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -3958,22 +3967,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MPG</t>
+          <t>Enterprise Products</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Blackcomb Spread 5</t>
+          <t>Texas City Tank Inspections</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/8f96hglr2igfibinjx7v6/AFSlCv7s3rz7q6mH4HKvQhE?rlkey=dpa02qv52p8ma0k3fpm6vgfon&amp;st=ti3xpyko&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/jbtud46rkg0652ukwaq08/ADUSamMzcIPopx_e1aIMeJo?rlkey=slnljxojww8nvxjcicwr9n26h&amp;st=mwghcpow&amp;dl=0</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>cpena@mpg-plc.com, lharrod@mpg-plc.com, isandlin@mpg-plc.com, patafoya@mpg-plc.com, bsanger@mpg-plc.com</t>
+          <t>bwott@eprod.com</t>
         </is>
       </c>
     </row>
@@ -3985,17 +3994,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Howard Energy OLU</t>
+          <t>Blackcomb Spread 5</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/fmept35wh6z03pnuyjjve/AABu6EMmGEc7kjFHsg1T9sg?rlkey=nu44grjidqjo4vv7szzr1v0o2&amp;st=ohec5e24&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/8f96hglr2igfibinjx7v6/AFSlCv7s3rz7q6mH4HKvQhE?rlkey=dpa02qv52p8ma0k3fpm6vgfon&amp;st=ti3xpyko&amp;dl=0</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>lharrod@mpg-plc.com, patafoya@mpg-plc.com, Mdenton@mpg-plc.com, rcaraveo@mpg-plc.com, klynn@mpg-plc.com</t>
+          <t>cpena@mpg-plc.com, lharrod@mpg-plc.com, isandlin@mpg-plc.com, patafoya@mpg-plc.com, bsanger@mpg-plc.com</t>
         </is>
       </c>
     </row>
@@ -4007,78 +4016,83 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Traverse</t>
+          <t>Howard Energy OLU</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/59s3fdlbvs6j1tq0ifwgr/ADt4bBu2DT-6SO1qklXlbu4?rlkey=sj1681fgfbchqrtks293lirk2&amp;st=c200hnzb&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/fmept35wh6z03pnuyjjve/AABu6EMmGEc7kjFHsg1T9sg?rlkey=nu44grjidqjo4vv7szzr1v0o2&amp;st=ohec5e24&amp;dl=0</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>cpena@mpg-plc.com, lharrod@mpg-plc.com, isandlin@mpg-plc.com, cwillie@mpg-plc.com, zfontenot@mpg-plc.com, bsanger@mpg-plc.com</t>
+          <t>lharrod@mpg-plc.com, patafoya@mpg-plc.com, Mdenton@mpg-plc.com, rcaraveo@mpg-plc.com, klynn@mpg-plc.com</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Sunland</t>
+          <t>MPG</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sempra LAS Facility</t>
+          <t>Traverse</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/vkuayzt15k8td7v3vgw1q/AG4CfYEs7hyVbMl0Oa-FQM4?rlkey=27hhbf0y1zz08n1s56h1vu6rh&amp;st=b4w57uc2&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/59s3fdlbvs6j1tq0ifwgr/ADt4bBu2DT-6SO1qklXlbu4?rlkey=sj1681fgfbchqrtks293lirk2&amp;st=c200hnzb&amp;dl=0</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>ccbelfour@sunlandconstruction.com, tjstamey@sunlandconstruction.com, kmward@sunlandconstruction.com, cjmanuel@sunlandconstruction.com, dttise@sunlandconstruction.com</t>
+          <t>cpena@mpg-plc.com, lharrod@mpg-plc.com, isandlin@mpg-plc.com, cwillie@mpg-plc.com, zfontenot@mpg-plc.com, bsanger@mpg-plc.com</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TEST</t>
+          <t>Sunland</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>TEST</t>
+          <t>Sempra LAS Facility</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/2u22rkfy8auzr19nq103s/AKCiHNTg1Lei6w9LW-Rrq0k?rlkey=bnrbpwsdjrb740q2tnlc3w34y&amp;st=bwn17cis&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/vkuayzt15k8td7v3vgw1q/AG4CfYEs7hyVbMl0Oa-FQM4?rlkey=27hhbf0y1zz08n1s56h1vu6rh&amp;st=b4w57uc2&amp;dl=0</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>smclaren@archaerial.com</t>
+          <t>ccbelfour@sunlandconstruction.com, tjstamey@sunlandconstruction.com, kmward@sunlandconstruction.com, cjmanuel@sunlandconstruction.com, dttise@sunlandconstruction.com</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Whitewater</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Blackcomb Midkiff Lateral</t>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/2u22rkfy8auzr19nq103s/AKCiHNTg1Lei6w9LW-Rrq0k?rlkey=bnrbpwsdjrb740q2tnlc3w34y&amp;st=bwn17cis&amp;dl=0</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>sfife@wwm-llc.com, zach@wwm-llc.com</t>
+          <t>smclaren@archaerial.com</t>
         </is>
       </c>
     </row>
@@ -4090,17 +4104,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Eiger</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/68n6e8pfm5766gb3peg2z/APMLs2RrSMAQsof6ZEnFB9M?rlkey=l3vawd6x5nbc0yn9utha6s9l4&amp;st=bgxydz50&amp;dl=0</t>
+          <t>Blackcomb Midkiff Lateral</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>lee@wwm-llc.com, eurbizu@wwm-llc.com, nick@wwm-llc.com</t>
+          <t>sfife@wwm-llc.com, zach@wwm-llc.com</t>
         </is>
       </c>
     </row>
@@ -4112,34 +4121,39 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Monahans Lateral</t>
+          <t>Eiger</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/qsig1qg2auszm47fab6gn/AJwovk21_a8KBBG1NCm46_c?rlkey=rmz9wzmw0jtwb5snydzz7nb6p&amp;st=3qodbo5v&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/68n6e8pfm5766gb3peg2z/APMLs2RrSMAQsof6ZEnFB9M?rlkey=l3vawd6x5nbc0yn9utha6s9l4&amp;st=bgxydz50&amp;dl=0</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>sfife@wwm-llc.com</t>
+          <t>lee@wwm-llc.com, eurbizu@wwm-llc.com, nick@wwm-llc.com</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Williams</t>
+          <t>Whitewater</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Mainline A</t>
+          <t>Monahans Lateral</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/qsig1qg2auszm47fab6gn/AJwovk21_a8KBBG1NCm46_c?rlkey=rmz9wzmw0jtwb5snydzz7nb6p&amp;st=3qodbo5v&amp;dl=0</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Mike.Smitherman@Williams.com, Roy.Guerrero@williams.com, Santos.Rocha@Williams.com, James.Mills@williams.com</t>
+          <t>sfife@wwm-llc.com</t>
         </is>
       </c>
     </row>
@@ -4151,12 +4165,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NOPI - 4 Mile Segment</t>
+          <t>Mainline A</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Mike.Smitherman@Williams.com, Roy.Guerrero@williams.com</t>
+          <t>Mike.Smitherman@Williams.com, Roy.Guerrero@williams.com, Santos.Rocha@Williams.com, James.Mills@williams.com</t>
         </is>
       </c>
     </row>
@@ -4168,12 +4182,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>NWC Gathering System</t>
+          <t>NOPI - 4 Mile Segment</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Daniel.young@williams.com</t>
+          <t>Mike.Smitherman@Williams.com, Roy.Guerrero@williams.com</t>
         </is>
       </c>
     </row>
@@ -4185,12 +4199,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Padres Island Pipeline</t>
+          <t>NWC Gathering System</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Mike.Smitherman@Williams.com, Roy.Guerrero@williams.com</t>
+          <t>Daniel.young@williams.com</t>
         </is>
       </c>
     </row>
@@ -4202,17 +4216,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Station 145</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>https://www.dropbox.com/scl/fo/z8kvz6pb2j2r09oo2c97g/AFQLt9GkR8taMaiVPmxvHh4?rlkey=4ts1b97rjx5lbe0br3fbc2wjf&amp;st=ru4xwzl3&amp;dl=0</t>
+          <t>Padres Island Pipeline</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>joshua.colombo@williams.com, james.a.raschke@williams.com, Jeff.King@Williams.com, jeff.l.gallimore@williams.com, Sam.Lawrence@Williams.com, Kevin.Murray@Williams.com, chad.dlugoszewski@williams.com, Philip.Giblin@williams.com, Michael.T.Barron@Williams.com, Austin.Justice@williams.com, timothy.petrea@williams.com</t>
+          <t>Mike.Smitherman@Williams.com, Roy.Guerrero@williams.com</t>
         </is>
       </c>
     </row>
@@ -4224,17 +4233,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Station 150</t>
+          <t>Station 145</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/kaxyjgx5dcjqozysedsvw/AGutILn_Cw8siidIM1J_vvI?rlkey=5mynmrgcc7fvyy35k3b8o1waq&amp;st=32gshoxy&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/z8kvz6pb2j2r09oo2c97g/AFQLt9GkR8taMaiVPmxvHh4?rlkey=4ts1b97rjx5lbe0br3fbc2wjf&amp;st=ru4xwzl3&amp;dl=0</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>leann.sprayberry@williams.com, steven.johnston@williams.com, ssluttersr@gmail.com, james.a.raschke@williams.com, bradley.george@williams.com, chad.dlugoszewski@williams.com, jeff.l.gallimore@williams.com, timothy.petrea@williams.com</t>
+          <t>joshua.colombo@williams.com, james.a.raschke@williams.com, Jeff.King@Williams.com, jeff.l.gallimore@williams.com, Sam.Lawrence@Williams.com, Kevin.Murray@Williams.com, chad.dlugoszewski@williams.com, Philip.Giblin@williams.com, Michael.T.Barron@Williams.com, Austin.Justice@williams.com, timothy.petrea@williams.com</t>
         </is>
       </c>
     </row>
@@ -4246,17 +4255,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Station 155</t>
+          <t>Station 150</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/m3ziycemltti4rntzjwxn/AAD0779D_F1HEl9iia9r07M?rlkey=2brdm1ebw4h6v4fx3gk0fbqvq&amp;st=4kae51wa&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/kaxyjgx5dcjqozysedsvw/AGutILn_Cw8siidIM1J_vvI?rlkey=5mynmrgcc7fvyy35k3b8o1waq&amp;st=32gshoxy&amp;dl=0</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>james.a.raschke@williams.com, leann.sprayberry@williams.com, steven.johnston@williams.com, ssluttersr@gmail.com, bradley.george@williams.com, keith.murray@williams.com, scott.emerson@williams.com</t>
+          <t>leann.sprayberry@williams.com, james.a.raschke@williams.com, bradley.george@williams.com, chad.dlugoszewski@williams.com, jeff.l.gallimore@williams.com, timothy.petrea@williams.com, Mike.Fitzpatrick@Williams.com</t>
         </is>
       </c>
     </row>
@@ -4268,12 +4277,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Station 160</t>
+          <t>Station 155</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.dropbox.com/scl/fo/83sgdjxpgsdrnqdv8srm3/ADhvHR96Uyk1p8Ii4cNtouA?rlkey=o7d5rrmbpg7tgmedpsmb6owny&amp;st=fl56lkhe&amp;dl=0</t>
+          <t>https://www.dropbox.com/scl/fo/m3ziycemltti4rntzjwxn/AAD0779D_F1HEl9iia9r07M?rlkey=2brdm1ebw4h6v4fx3gk0fbqvq&amp;st=4kae51wa&amp;dl=0</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4290,15 +4299,37 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>Station 160</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fo/83sgdjxpgsdrnqdv8srm3/ADhvHR96Uyk1p8Ii4cNtouA?rlkey=o7d5rrmbpg7tgmedpsmb6owny&amp;st=fl56lkhe&amp;dl=0</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>james.a.raschke@williams.com, leann.sprayberry@williams.com, steven.johnston@williams.com, ssluttersr@gmail.com, bradley.george@williams.com, keith.murray@williams.com, scott.emerson@williams.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Williams</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>Station 165</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>https://www.dropbox.com/scl/fo/7e1548qjcwrxwufynwox3/ANTe2IBK5ChXU-pU8cg42A8?rlkey=n023itk90g2p7tflky6pnp3os&amp;st=oz50awuz&amp;dl=0</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>joshua.colombo@williams.com, roddy.a.ballard@williams.com, bill.bates@williams.com, Sam.Lawrence@Williams.com, Kevin.Murray@Williams.com, David.LaRue@williams.com, Sandra.Hamilton@williams.com</t>
         </is>
@@ -4352,7 +4383,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>

</xml_diff>